<commit_message>
Please provide the file changes (diffs) so I can generate a commit message.
</commit_message>
<xml_diff>
--- a/OI/jeu_du_kanban/clé USB Jeu du Kanban/Consommables/Documents.xlsx
+++ b/OI/jeu_du_kanban/clé USB Jeu du Kanban/Consommables/Documents.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/Jeu du KANBAN/clé USB Jeu du Kanban/Consommables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/jeu_du_kanban/clé USB Jeu du Kanban/Consommables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_77B6C54FE39E7C3E24E1221787039D3B0B441E73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B89F87C-970E-446C-A834-B1DA08050A03}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="11_77B6C54FE39E7C3E24E1221787039D3B0B441E73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE2E8644-6C3E-4205-B03B-FE124A6ACBFB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="830" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="830" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuille de suivi" sheetId="4" r:id="rId1"/>
@@ -1680,15 +1680,75 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
@@ -1713,65 +1773,11 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1800,6 +1806,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1827,40 +1866,28 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1869,30 +1896,9 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1916,12 +1922,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -11813,6 +11813,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
@@ -12180,7 +12184,7 @@
       <c r="A2" s="167" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="189"/>
+      <c r="B2" s="168"/>
       <c r="C2" s="165"/>
       <c r="D2" s="165"/>
       <c r="E2" s="166"/>
@@ -12188,7 +12192,7 @@
         <v>92</v>
       </c>
       <c r="H2" s="25"/>
-      <c r="J2" s="170" t="s">
+      <c r="J2" s="181" t="s">
         <v>93</v>
       </c>
       <c r="K2" s="165"/>
@@ -12208,7 +12212,7 @@
       </c>
     </row>
     <row r="3" spans="1:19" ht="14.25" customHeight="1">
-      <c r="O3" s="175" t="s">
+      <c r="O3" s="195" t="s">
         <v>19</v>
       </c>
       <c r="P3" s="4"/>
@@ -12217,7 +12221,7 @@
       <c r="S3" s="5"/>
     </row>
     <row r="4" spans="1:19" ht="14.25" customHeight="1" thickBot="1">
-      <c r="O4" s="175"/>
+      <c r="O4" s="195"/>
       <c r="P4" s="4"/>
       <c r="Q4" s="3"/>
       <c r="R4" s="3"/>
@@ -12227,105 +12231,105 @@
       <c r="H5" s="167" t="s">
         <v>89</v>
       </c>
-      <c r="I5" s="168"/>
-      <c r="J5" s="169"/>
-      <c r="O5" s="175"/>
+      <c r="I5" s="176"/>
+      <c r="J5" s="177"/>
+      <c r="O5" s="195"/>
       <c r="P5" s="4"/>
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="S5" s="5"/>
     </row>
     <row r="6" spans="1:19" ht="14.25" customHeight="1">
-      <c r="H6" s="183" t="s">
+      <c r="H6" s="185" t="s">
         <v>7</v>
       </c>
-      <c r="I6" s="186" t="s">
+      <c r="I6" s="188" t="s">
         <v>87</v>
       </c>
-      <c r="J6" s="180" t="s">
+      <c r="J6" s="182" t="s">
         <v>1</v>
       </c>
-      <c r="K6" s="171" t="s">
+      <c r="K6" s="191" t="s">
         <v>88</v>
       </c>
-      <c r="O6" s="175"/>
+      <c r="O6" s="195"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
       <c r="S6" s="5"/>
     </row>
     <row r="7" spans="1:19" ht="14.25" customHeight="1">
-      <c r="H7" s="184"/>
-      <c r="I7" s="187"/>
-      <c r="J7" s="181"/>
-      <c r="K7" s="171"/>
-      <c r="O7" s="175"/>
+      <c r="H7" s="186"/>
+      <c r="I7" s="189"/>
+      <c r="J7" s="183"/>
+      <c r="K7" s="191"/>
+      <c r="O7" s="195"/>
       <c r="P7" s="4"/>
       <c r="Q7" s="3"/>
       <c r="R7" s="3"/>
       <c r="S7" s="5"/>
     </row>
     <row r="8" spans="1:19" ht="14.25" customHeight="1">
-      <c r="H8" s="184"/>
-      <c r="I8" s="187"/>
-      <c r="J8" s="181"/>
-      <c r="K8" s="171"/>
-      <c r="O8" s="175"/>
+      <c r="H8" s="186"/>
+      <c r="I8" s="189"/>
+      <c r="J8" s="183"/>
+      <c r="K8" s="191"/>
+      <c r="O8" s="195"/>
       <c r="P8" s="4"/>
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
       <c r="S8" s="5"/>
     </row>
     <row r="9" spans="1:19" ht="14.25" customHeight="1">
-      <c r="H9" s="184"/>
-      <c r="I9" s="187"/>
-      <c r="J9" s="181"/>
-      <c r="K9" s="171"/>
-      <c r="M9" s="173" t="s">
+      <c r="H9" s="186"/>
+      <c r="I9" s="189"/>
+      <c r="J9" s="183"/>
+      <c r="K9" s="191"/>
+      <c r="M9" s="193" t="s">
         <v>18</v>
       </c>
-      <c r="N9" s="173"/>
-      <c r="O9" s="173"/>
+      <c r="N9" s="193"/>
+      <c r="O9" s="193"/>
       <c r="P9" s="4"/>
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
       <c r="S9" s="5"/>
     </row>
     <row r="10" spans="1:19" ht="14.25" customHeight="1" thickBot="1">
-      <c r="B10" s="190" t="s">
+      <c r="B10" s="169" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="190"/>
-      <c r="D10" s="190"/>
-      <c r="E10" s="190"/>
-      <c r="F10" s="190"/>
-      <c r="G10" s="190"/>
-      <c r="H10" s="184"/>
-      <c r="I10" s="187"/>
-      <c r="J10" s="181"/>
-      <c r="K10" s="171"/>
-      <c r="M10" s="173"/>
-      <c r="N10" s="173"/>
-      <c r="O10" s="173"/>
+      <c r="C10" s="169"/>
+      <c r="D10" s="169"/>
+      <c r="E10" s="169"/>
+      <c r="F10" s="169"/>
+      <c r="G10" s="169"/>
+      <c r="H10" s="186"/>
+      <c r="I10" s="189"/>
+      <c r="J10" s="183"/>
+      <c r="K10" s="191"/>
+      <c r="M10" s="193"/>
+      <c r="N10" s="193"/>
+      <c r="O10" s="193"/>
       <c r="P10" s="8"/>
       <c r="Q10" s="9"/>
       <c r="R10" s="9"/>
       <c r="S10" s="10"/>
     </row>
     <row r="11" spans="1:19" ht="6" customHeight="1" thickBot="1">
-      <c r="B11" s="190"/>
-      <c r="C11" s="190"/>
-      <c r="D11" s="190"/>
-      <c r="E11" s="190"/>
-      <c r="F11" s="190"/>
-      <c r="G11" s="190"/>
-      <c r="H11" s="184"/>
-      <c r="I11" s="187"/>
-      <c r="J11" s="181"/>
-      <c r="K11" s="171"/>
-      <c r="M11" s="174"/>
-      <c r="N11" s="174"/>
-      <c r="O11" s="174"/>
+      <c r="B11" s="169"/>
+      <c r="C11" s="169"/>
+      <c r="D11" s="169"/>
+      <c r="E11" s="169"/>
+      <c r="F11" s="169"/>
+      <c r="G11" s="169"/>
+      <c r="H11" s="186"/>
+      <c r="I11" s="189"/>
+      <c r="J11" s="183"/>
+      <c r="K11" s="191"/>
+      <c r="M11" s="194"/>
+      <c r="N11" s="194"/>
+      <c r="O11" s="194"/>
     </row>
     <row r="12" spans="1:19" ht="18" customHeight="1" thickBot="1">
       <c r="A12" s="19" t="s">
@@ -12337,10 +12341,10 @@
       <c r="E12" s="120"/>
       <c r="F12" s="120"/>
       <c r="G12" s="122"/>
-      <c r="H12" s="185"/>
-      <c r="I12" s="188"/>
-      <c r="J12" s="182"/>
-      <c r="K12" s="171"/>
+      <c r="H12" s="187"/>
+      <c r="I12" s="190"/>
+      <c r="J12" s="184"/>
+      <c r="K12" s="191"/>
       <c r="L12" s="12"/>
       <c r="M12" s="30" t="s">
         <v>8</v>
@@ -13165,10 +13169,10 @@
       <c r="S44" s="14"/>
     </row>
     <row r="45" spans="1:20" ht="21" customHeight="1" thickBot="1">
-      <c r="F45" s="196" t="s">
+      <c r="F45" s="175" t="s">
         <v>91</v>
       </c>
-      <c r="G45" s="196"/>
+      <c r="G45" s="175"/>
       <c r="H45" s="6"/>
       <c r="I45" s="7"/>
       <c r="J45" s="25"/>
@@ -13198,23 +13202,23 @@
       <c r="C47" s="121"/>
       <c r="D47" s="121"/>
       <c r="E47" s="121"/>
-      <c r="F47" s="197" t="s">
+      <c r="F47" s="178" t="s">
         <v>15</v>
       </c>
-      <c r="G47" s="198"/>
+      <c r="G47" s="179"/>
       <c r="H47" s="167"/>
-      <c r="I47" s="168"/>
-      <c r="J47" s="169"/>
+      <c r="I47" s="176"/>
+      <c r="J47" s="177"/>
       <c r="L47" s="11"/>
       <c r="M47" s="2"/>
       <c r="N47" s="2"/>
       <c r="O47" s="167"/>
-      <c r="P47" s="168"/>
-      <c r="Q47" s="169"/>
-      <c r="R47" s="172" t="s">
+      <c r="P47" s="176"/>
+      <c r="Q47" s="177"/>
+      <c r="R47" s="192" t="s">
         <v>16</v>
       </c>
-      <c r="S47" s="172"/>
+      <c r="S47" s="192"/>
       <c r="T47" s="11"/>
     </row>
     <row r="48" spans="1:20" ht="10.5" customHeight="1" thickBot="1">
@@ -13230,25 +13234,25 @@
       <c r="B49" s="118"/>
       <c r="C49" s="118"/>
       <c r="D49" s="118"/>
-      <c r="E49" s="194" t="s">
+      <c r="E49" s="173" t="s">
         <v>90</v>
       </c>
-      <c r="F49" s="194"/>
-      <c r="G49" s="195"/>
-      <c r="H49" s="191">
+      <c r="F49" s="173"/>
+      <c r="G49" s="174"/>
+      <c r="H49" s="170">
         <v>32</v>
       </c>
-      <c r="I49" s="192"/>
-      <c r="J49" s="193"/>
+      <c r="I49" s="171"/>
+      <c r="J49" s="172"/>
       <c r="K49" s="23"/>
       <c r="M49" s="23"/>
-      <c r="O49" s="176"/>
-      <c r="P49" s="177"/>
-      <c r="Q49" s="178"/>
-      <c r="R49" s="172" t="s">
+      <c r="O49" s="196"/>
+      <c r="P49" s="197"/>
+      <c r="Q49" s="198"/>
+      <c r="R49" s="192" t="s">
         <v>17</v>
       </c>
-      <c r="S49" s="172"/>
+      <c r="S49" s="192"/>
       <c r="T49" s="11"/>
     </row>
     <row r="50" spans="1:20" ht="10.5" customHeight="1" thickBot="1">
@@ -13270,22 +13274,22 @@
       <c r="C51" s="118"/>
       <c r="D51" s="118"/>
       <c r="E51" s="118"/>
-      <c r="F51" s="179" t="s">
+      <c r="F51" s="180" t="s">
         <v>40</v>
       </c>
-      <c r="G51" s="179"/>
+      <c r="G51" s="180"/>
       <c r="H51" s="167"/>
-      <c r="I51" s="168"/>
-      <c r="J51" s="169"/>
+      <c r="I51" s="176"/>
+      <c r="J51" s="177"/>
       <c r="K51" s="118"/>
       <c r="L51" s="117"/>
-      <c r="O51" s="170"/>
+      <c r="O51" s="181"/>
       <c r="P51" s="165"/>
       <c r="Q51" s="166"/>
-      <c r="R51" s="172" t="s">
+      <c r="R51" s="192" t="s">
         <v>0</v>
       </c>
-      <c r="S51" s="172"/>
+      <c r="S51" s="192"/>
     </row>
     <row r="52" spans="1:20" ht="18" customHeight="1">
       <c r="R52" s="26"/>
@@ -13312,21 +13316,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B10:G11"/>
-    <mergeCell ref="H49:J49"/>
-    <mergeCell ref="E49:G49"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="H47:J47"/>
-    <mergeCell ref="F51:G51"/>
-    <mergeCell ref="H51:J51"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="J6:J12"/>
-    <mergeCell ref="H6:H12"/>
-    <mergeCell ref="I6:I12"/>
     <mergeCell ref="L2:M2"/>
     <mergeCell ref="O47:Q47"/>
     <mergeCell ref="O51:Q51"/>
@@ -13337,6 +13326,21 @@
     <mergeCell ref="R51:S51"/>
     <mergeCell ref="R49:S49"/>
     <mergeCell ref="O49:Q49"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="H51:J51"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="J6:J12"/>
+    <mergeCell ref="H6:H12"/>
+    <mergeCell ref="I6:I12"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="B10:G11"/>
+    <mergeCell ref="H49:J49"/>
+    <mergeCell ref="E49:G49"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="H47:J47"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.47244094488188981" right="0.47244094488188981" top="0.78740157480314965" bottom="0.78740157480314965" header="0.51181102362204722" footer="0.51181102362204722"/>
@@ -13374,7 +13378,7 @@
       <c r="A2" s="167" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="189"/>
+      <c r="B2" s="168"/>
       <c r="C2" s="165" t="s">
         <v>49</v>
       </c>
@@ -13386,14 +13390,14 @@
       <c r="H2" s="25">
         <v>1</v>
       </c>
-      <c r="J2" s="170" t="s">
+      <c r="J2" s="181" t="s">
         <v>93</v>
       </c>
       <c r="K2" s="165"/>
-      <c r="L2" s="199">
+      <c r="L2" s="201">
         <v>3</v>
       </c>
-      <c r="M2" s="200"/>
+      <c r="M2" s="202"/>
       <c r="P2" s="20" t="s">
         <v>3</v>
       </c>
@@ -13408,7 +13412,7 @@
       </c>
     </row>
     <row r="3" spans="1:19" ht="14.25" customHeight="1">
-      <c r="O3" s="175" t="s">
+      <c r="O3" s="195" t="s">
         <v>19</v>
       </c>
       <c r="P3" s="4">
@@ -13425,7 +13429,7 @@
       </c>
     </row>
     <row r="4" spans="1:19" ht="14.25" customHeight="1" thickBot="1">
-      <c r="O4" s="175"/>
+      <c r="O4" s="195"/>
       <c r="P4" s="4">
         <v>2</v>
       </c>
@@ -13443,9 +13447,9 @@
       <c r="H5" s="167" t="s">
         <v>89</v>
       </c>
-      <c r="I5" s="168"/>
-      <c r="J5" s="169"/>
-      <c r="O5" s="175"/>
+      <c r="I5" s="176"/>
+      <c r="J5" s="177"/>
+      <c r="O5" s="195"/>
       <c r="P5" s="4">
         <v>3</v>
       </c>
@@ -13460,96 +13464,96 @@
       </c>
     </row>
     <row r="6" spans="1:19" ht="14.25" customHeight="1">
-      <c r="H6" s="183" t="s">
+      <c r="H6" s="185" t="s">
         <v>7</v>
       </c>
-      <c r="I6" s="186" t="s">
+      <c r="I6" s="188" t="s">
         <v>87</v>
       </c>
-      <c r="J6" s="180" t="s">
+      <c r="J6" s="182" t="s">
         <v>1</v>
       </c>
-      <c r="K6" s="171" t="s">
+      <c r="K6" s="191" t="s">
         <v>88</v>
       </c>
-      <c r="O6" s="175"/>
+      <c r="O6" s="195"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
       <c r="S6" s="5"/>
     </row>
     <row r="7" spans="1:19" ht="14.25" customHeight="1">
-      <c r="H7" s="184"/>
-      <c r="I7" s="187"/>
-      <c r="J7" s="181"/>
-      <c r="K7" s="171"/>
-      <c r="O7" s="175"/>
+      <c r="H7" s="186"/>
+      <c r="I7" s="189"/>
+      <c r="J7" s="183"/>
+      <c r="K7" s="191"/>
+      <c r="O7" s="195"/>
       <c r="P7" s="4"/>
       <c r="Q7" s="3"/>
       <c r="R7" s="3"/>
       <c r="S7" s="5"/>
     </row>
     <row r="8" spans="1:19" ht="14.25" customHeight="1">
-      <c r="H8" s="184"/>
-      <c r="I8" s="187"/>
-      <c r="J8" s="181"/>
-      <c r="K8" s="171"/>
-      <c r="O8" s="175"/>
+      <c r="H8" s="186"/>
+      <c r="I8" s="189"/>
+      <c r="J8" s="183"/>
+      <c r="K8" s="191"/>
+      <c r="O8" s="195"/>
       <c r="P8" s="4"/>
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
       <c r="S8" s="5"/>
     </row>
     <row r="9" spans="1:19" ht="14.25" customHeight="1">
-      <c r="H9" s="184"/>
-      <c r="I9" s="187"/>
-      <c r="J9" s="181"/>
-      <c r="K9" s="171"/>
-      <c r="M9" s="173" t="s">
+      <c r="H9" s="186"/>
+      <c r="I9" s="189"/>
+      <c r="J9" s="183"/>
+      <c r="K9" s="191"/>
+      <c r="M9" s="193" t="s">
         <v>18</v>
       </c>
-      <c r="N9" s="173"/>
-      <c r="O9" s="173"/>
+      <c r="N9" s="193"/>
+      <c r="O9" s="193"/>
       <c r="P9" s="4"/>
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
       <c r="S9" s="5"/>
     </row>
     <row r="10" spans="1:19" ht="14.25" customHeight="1" thickBot="1">
-      <c r="B10" s="190" t="s">
+      <c r="B10" s="169" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="190"/>
-      <c r="D10" s="190"/>
-      <c r="E10" s="190"/>
-      <c r="F10" s="190"/>
-      <c r="G10" s="190"/>
-      <c r="H10" s="184"/>
-      <c r="I10" s="187"/>
-      <c r="J10" s="181"/>
-      <c r="K10" s="171"/>
-      <c r="M10" s="173"/>
-      <c r="N10" s="173"/>
-      <c r="O10" s="173"/>
+      <c r="C10" s="169"/>
+      <c r="D10" s="169"/>
+      <c r="E10" s="169"/>
+      <c r="F10" s="169"/>
+      <c r="G10" s="169"/>
+      <c r="H10" s="186"/>
+      <c r="I10" s="189"/>
+      <c r="J10" s="183"/>
+      <c r="K10" s="191"/>
+      <c r="M10" s="193"/>
+      <c r="N10" s="193"/>
+      <c r="O10" s="193"/>
       <c r="P10" s="8"/>
       <c r="Q10" s="9"/>
       <c r="R10" s="9"/>
       <c r="S10" s="10"/>
     </row>
     <row r="11" spans="1:19" ht="6" customHeight="1" thickBot="1">
-      <c r="B11" s="190"/>
-      <c r="C11" s="190"/>
-      <c r="D11" s="190"/>
-      <c r="E11" s="190"/>
-      <c r="F11" s="190"/>
-      <c r="G11" s="190"/>
-      <c r="H11" s="184"/>
-      <c r="I11" s="187"/>
-      <c r="J11" s="181"/>
-      <c r="K11" s="171"/>
-      <c r="M11" s="174"/>
-      <c r="N11" s="174"/>
-      <c r="O11" s="174"/>
+      <c r="B11" s="169"/>
+      <c r="C11" s="169"/>
+      <c r="D11" s="169"/>
+      <c r="E11" s="169"/>
+      <c r="F11" s="169"/>
+      <c r="G11" s="169"/>
+      <c r="H11" s="186"/>
+      <c r="I11" s="189"/>
+      <c r="J11" s="183"/>
+      <c r="K11" s="191"/>
+      <c r="M11" s="194"/>
+      <c r="N11" s="194"/>
+      <c r="O11" s="194"/>
     </row>
     <row r="12" spans="1:19" ht="18" customHeight="1" thickBot="1">
       <c r="A12" s="19" t="s">
@@ -13565,10 +13569,10 @@
       <c r="E12" s="120"/>
       <c r="F12" s="120"/>
       <c r="G12" s="122"/>
-      <c r="H12" s="185"/>
-      <c r="I12" s="188"/>
-      <c r="J12" s="182"/>
-      <c r="K12" s="171"/>
+      <c r="H12" s="187"/>
+      <c r="I12" s="190"/>
+      <c r="J12" s="184"/>
+      <c r="K12" s="191"/>
       <c r="L12" s="12"/>
       <c r="M12" s="30" t="s">
         <v>8</v>
@@ -14397,10 +14401,10 @@
       <c r="S44" s="14"/>
     </row>
     <row r="45" spans="1:20" ht="21" customHeight="1" thickBot="1">
-      <c r="F45" s="196" t="s">
+      <c r="F45" s="175" t="s">
         <v>91</v>
       </c>
-      <c r="G45" s="196"/>
+      <c r="G45" s="175"/>
       <c r="H45" s="134">
         <v>6</v>
       </c>
@@ -14440,27 +14444,27 @@
       <c r="C47" s="121"/>
       <c r="D47" s="121"/>
       <c r="E47" s="121"/>
-      <c r="F47" s="197" t="s">
+      <c r="F47" s="178" t="s">
         <v>15</v>
       </c>
-      <c r="G47" s="198"/>
-      <c r="H47" s="191">
+      <c r="G47" s="179"/>
+      <c r="H47" s="170">
         <v>8</v>
       </c>
-      <c r="I47" s="192"/>
-      <c r="J47" s="193"/>
+      <c r="I47" s="171"/>
+      <c r="J47" s="172"/>
       <c r="L47" s="11"/>
       <c r="M47" s="2"/>
       <c r="N47" s="2"/>
       <c r="O47" s="167">
         <v>3</v>
       </c>
-      <c r="P47" s="168"/>
-      <c r="Q47" s="169"/>
-      <c r="R47" s="172" t="s">
+      <c r="P47" s="176"/>
+      <c r="Q47" s="177"/>
+      <c r="R47" s="192" t="s">
         <v>16</v>
       </c>
-      <c r="S47" s="172"/>
+      <c r="S47" s="192"/>
       <c r="T47" s="11"/>
     </row>
     <row r="48" spans="1:20" ht="10.5" customHeight="1" thickBot="1">
@@ -14476,28 +14480,28 @@
       <c r="B49" s="118"/>
       <c r="C49" s="118"/>
       <c r="D49" s="118"/>
-      <c r="E49" s="194" t="s">
+      <c r="E49" s="173" t="s">
         <v>90</v>
       </c>
-      <c r="F49" s="194"/>
-      <c r="G49" s="195"/>
-      <c r="H49" s="191">
+      <c r="F49" s="173"/>
+      <c r="G49" s="174"/>
+      <c r="H49" s="170">
         <v>32</v>
       </c>
-      <c r="I49" s="192"/>
-      <c r="J49" s="193"/>
+      <c r="I49" s="171"/>
+      <c r="J49" s="172"/>
       <c r="K49" s="23"/>
       <c r="M49" s="23"/>
-      <c r="O49" s="176">
+      <c r="O49" s="196">
         <v>34</v>
       </c>
-      <c r="P49" s="177"/>
-      <c r="Q49" s="178"/>
-      <c r="R49" s="247" t="s">
+      <c r="P49" s="197"/>
+      <c r="Q49" s="198"/>
+      <c r="R49" s="199" t="s">
         <v>114</v>
       </c>
-      <c r="S49" s="248"/>
-      <c r="T49" s="248"/>
+      <c r="S49" s="200"/>
+      <c r="T49" s="200"/>
     </row>
     <row r="50" spans="1:20" ht="10.5" customHeight="1" thickBot="1">
       <c r="B50" s="118"/>
@@ -14518,28 +14522,28 @@
       <c r="C51" s="118"/>
       <c r="D51" s="118"/>
       <c r="E51" s="118"/>
-      <c r="F51" s="179" t="s">
+      <c r="F51" s="180" t="s">
         <v>40</v>
       </c>
-      <c r="G51" s="179"/>
-      <c r="H51" s="201">
+      <c r="G51" s="180"/>
+      <c r="H51" s="203">
         <f>24/32</f>
         <v>0.75</v>
       </c>
-      <c r="I51" s="202"/>
-      <c r="J51" s="203"/>
+      <c r="I51" s="204"/>
+      <c r="J51" s="205"/>
       <c r="K51" s="118"/>
       <c r="L51" s="117"/>
-      <c r="O51" s="201">
+      <c r="O51" s="203">
         <f>(O49-O47)/O49</f>
         <v>0.91176470588235292</v>
       </c>
-      <c r="P51" s="202"/>
-      <c r="Q51" s="203"/>
-      <c r="R51" s="172" t="s">
+      <c r="P51" s="204"/>
+      <c r="Q51" s="205"/>
+      <c r="R51" s="192" t="s">
         <v>0</v>
       </c>
-      <c r="S51" s="172"/>
+      <c r="S51" s="192"/>
     </row>
     <row r="52" spans="1:20" ht="18" customHeight="1">
       <c r="R52" s="26"/>
@@ -14566,12 +14570,15 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="R47:S47"/>
-    <mergeCell ref="M9:O11"/>
-    <mergeCell ref="O3:O8"/>
-    <mergeCell ref="R51:S51"/>
-    <mergeCell ref="O49:Q49"/>
-    <mergeCell ref="R49:T49"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="B10:G11"/>
+    <mergeCell ref="H49:J49"/>
+    <mergeCell ref="E49:G49"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="H47:J47"/>
     <mergeCell ref="L2:M2"/>
     <mergeCell ref="O47:Q47"/>
     <mergeCell ref="O51:Q51"/>
@@ -14582,15 +14589,12 @@
     <mergeCell ref="J6:J12"/>
     <mergeCell ref="H6:H12"/>
     <mergeCell ref="I6:I12"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B10:G11"/>
-    <mergeCell ref="H49:J49"/>
-    <mergeCell ref="E49:G49"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="H47:J47"/>
+    <mergeCell ref="R47:S47"/>
+    <mergeCell ref="M9:O11"/>
+    <mergeCell ref="O3:O8"/>
+    <mergeCell ref="R51:S51"/>
+    <mergeCell ref="O49:Q49"/>
+    <mergeCell ref="R49:T49"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.47244094488188981" right="0.47244094488188981" top="0.78740157480314965" bottom="0.78740157480314965" header="0.51181102362204722" footer="0.51181102362204722"/>
@@ -14649,7 +14653,7 @@
       <c r="M2" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="204" t="s">
+      <c r="O2" s="206" t="s">
         <v>55</v>
       </c>
     </row>
@@ -14664,7 +14668,7 @@
       <c r="J3" s="2"/>
       <c r="K3" s="50"/>
       <c r="M3" s="51"/>
-      <c r="O3" s="204"/>
+      <c r="O3" s="206"/>
     </row>
     <row r="4" spans="1:15">
       <c r="C4" s="2"/>
@@ -14676,10 +14680,10 @@
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
-      <c r="O4" s="205"/>
+      <c r="O4" s="207"/>
     </row>
     <row r="5" spans="1:15" ht="27" customHeight="1">
-      <c r="A5" s="207" t="s">
+      <c r="A5" s="209" t="s">
         <v>49</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -14697,7 +14701,7 @@
       <c r="O5" s="53"/>
     </row>
     <row r="6" spans="1:15">
-      <c r="A6" s="207"/>
+      <c r="A6" s="209"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -14710,7 +14714,7 @@
       <c r="K6" s="2"/>
     </row>
     <row r="7" spans="1:15" ht="27" customHeight="1">
-      <c r="A7" s="207"/>
+      <c r="A7" s="209"/>
       <c r="B7" s="2" t="s">
         <v>20</v>
       </c>
@@ -14739,7 +14743,7 @@
       <c r="K8" s="2"/>
     </row>
     <row r="9" spans="1:15" ht="27" customHeight="1">
-      <c r="A9" s="207" t="s">
+      <c r="A9" s="209" t="s">
         <v>50</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -14757,7 +14761,7 @@
       <c r="O9" s="53"/>
     </row>
     <row r="10" spans="1:15">
-      <c r="A10" s="207"/>
+      <c r="A10" s="209"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -14770,7 +14774,7 @@
       <c r="K10" s="2"/>
     </row>
     <row r="11" spans="1:15" ht="27" customHeight="1">
-      <c r="A11" s="207"/>
+      <c r="A11" s="209"/>
       <c r="B11" s="2" t="s">
         <v>113</v>
       </c>
@@ -14799,7 +14803,7 @@
       <c r="K12" s="2"/>
     </row>
     <row r="13" spans="1:15" ht="27" customHeight="1">
-      <c r="A13" s="207" t="s">
+      <c r="A13" s="209" t="s">
         <v>58</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -14817,7 +14821,7 @@
       <c r="O13" s="53"/>
     </row>
     <row r="14" spans="1:15">
-      <c r="A14" s="207"/>
+      <c r="A14" s="209"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -14830,7 +14834,7 @@
       <c r="K14" s="2"/>
     </row>
     <row r="15" spans="1:15" ht="27" customHeight="1">
-      <c r="A15" s="207"/>
+      <c r="A15" s="209"/>
       <c r="B15" s="2" t="s">
         <v>57</v>
       </c>
@@ -14846,7 +14850,7 @@
       <c r="O15" s="53"/>
     </row>
     <row r="16" spans="1:15">
-      <c r="A16" s="207"/>
+      <c r="A16" s="209"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
@@ -14859,7 +14863,7 @@
       <c r="K16" s="2"/>
     </row>
     <row r="17" spans="1:15" ht="27" customHeight="1">
-      <c r="A17" s="207"/>
+      <c r="A17" s="209"/>
       <c r="B17" s="2" t="s">
         <v>56</v>
       </c>
@@ -14907,15 +14911,15 @@
         <v>60</v>
       </c>
       <c r="G20" s="53"/>
-      <c r="I20" s="206" t="s">
+      <c r="I20" s="208" t="s">
         <v>97</v>
       </c>
-      <c r="J20" s="206"/>
-      <c r="K20" s="206"/>
-      <c r="L20" s="206"/>
-      <c r="M20" s="206"/>
-      <c r="N20" s="206"/>
-      <c r="O20" s="206"/>
+      <c r="J20" s="208"/>
+      <c r="K20" s="208"/>
+      <c r="L20" s="208"/>
+      <c r="M20" s="208"/>
+      <c r="N20" s="208"/>
+      <c r="O20" s="208"/>
     </row>
     <row r="21" spans="1:15" ht="42" customHeight="1">
       <c r="C21" s="55" t="s">
@@ -14929,13 +14933,13 @@
       <c r="G21" s="49" t="s">
         <v>63</v>
       </c>
-      <c r="I21" s="206"/>
-      <c r="J21" s="206"/>
-      <c r="K21" s="206"/>
-      <c r="L21" s="206"/>
-      <c r="M21" s="206"/>
-      <c r="N21" s="206"/>
-      <c r="O21" s="206"/>
+      <c r="I21" s="208"/>
+      <c r="J21" s="208"/>
+      <c r="K21" s="208"/>
+      <c r="L21" s="208"/>
+      <c r="M21" s="208"/>
+      <c r="N21" s="208"/>
+      <c r="O21" s="208"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -15004,7 +15008,7 @@
       <c r="M2" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="204" t="s">
+      <c r="O2" s="206" t="s">
         <v>55</v>
       </c>
     </row>
@@ -15032,7 +15036,7 @@
       <c r="M3" s="58">
         <v>3</v>
       </c>
-      <c r="O3" s="204"/>
+      <c r="O3" s="206"/>
     </row>
     <row r="4" spans="1:15" ht="15">
       <c r="C4" s="59"/>
@@ -15046,10 +15050,10 @@
       <c r="K4" s="59"/>
       <c r="L4" s="60"/>
       <c r="M4" s="60"/>
-      <c r="O4" s="205"/>
+      <c r="O4" s="207"/>
     </row>
     <row r="5" spans="1:15" ht="27" customHeight="1">
-      <c r="A5" s="207" t="s">
+      <c r="A5" s="209" t="s">
         <v>49</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -15082,7 +15086,7 @@
       </c>
     </row>
     <row r="6" spans="1:15" ht="15">
-      <c r="A6" s="207"/>
+      <c r="A6" s="209"/>
       <c r="B6" s="2"/>
       <c r="C6" s="59"/>
       <c r="D6" s="59"/>
@@ -15099,7 +15103,7 @@
       <c r="O6" s="60"/>
     </row>
     <row r="7" spans="1:15" ht="27" customHeight="1">
-      <c r="A7" s="207"/>
+      <c r="A7" s="209"/>
       <c r="B7" s="2" t="s">
         <v>20</v>
       </c>
@@ -15146,7 +15150,7 @@
       <c r="O8" s="60"/>
     </row>
     <row r="9" spans="1:15" ht="27" customHeight="1">
-      <c r="A9" s="207" t="s">
+      <c r="A9" s="209" t="s">
         <v>50</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -15182,7 +15186,7 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="15">
-      <c r="A10" s="207"/>
+      <c r="A10" s="209"/>
       <c r="B10" s="2"/>
       <c r="C10" s="59"/>
       <c r="D10" s="59"/>
@@ -15199,7 +15203,7 @@
       <c r="O10" s="60"/>
     </row>
     <row r="11" spans="1:15" ht="27" customHeight="1">
-      <c r="A11" s="207"/>
+      <c r="A11" s="209"/>
       <c r="B11" s="2" t="s">
         <v>113</v>
       </c>
@@ -15243,7 +15247,7 @@
       <c r="O12" s="60"/>
     </row>
     <row r="13" spans="1:15" ht="27" customHeight="1">
-      <c r="A13" s="207" t="s">
+      <c r="A13" s="209" t="s">
         <v>58</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -15273,7 +15277,7 @@
       </c>
     </row>
     <row r="14" spans="1:15" ht="15">
-      <c r="A14" s="207"/>
+      <c r="A14" s="209"/>
       <c r="B14" s="2"/>
       <c r="C14" s="59"/>
       <c r="D14" s="59"/>
@@ -15290,7 +15294,7 @@
       <c r="O14" s="60"/>
     </row>
     <row r="15" spans="1:15" ht="27" customHeight="1">
-      <c r="A15" s="207"/>
+      <c r="A15" s="209"/>
       <c r="B15" s="2" t="s">
         <v>57</v>
       </c>
@@ -15318,7 +15322,7 @@
       </c>
     </row>
     <row r="16" spans="1:15" ht="15">
-      <c r="A16" s="207"/>
+      <c r="A16" s="209"/>
       <c r="B16" s="2"/>
       <c r="C16" s="59"/>
       <c r="D16" s="59"/>
@@ -15335,7 +15339,7 @@
       <c r="O16" s="60"/>
     </row>
     <row r="17" spans="1:15" ht="27" customHeight="1">
-      <c r="A17" s="207"/>
+      <c r="A17" s="209"/>
       <c r="B17" s="2" t="s">
         <v>56</v>
       </c>
@@ -15450,12 +15454,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="16.5" customHeight="1">
-      <c r="A1" s="211" t="s">
+      <c r="A1" s="224" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="212"/>
-      <c r="C1" s="208"/>
-      <c r="D1" s="209"/>
+      <c r="B1" s="225"/>
+      <c r="C1" s="221"/>
+      <c r="D1" s="222"/>
       <c r="E1" s="140"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
@@ -15487,37 +15491,37 @@
     </row>
     <row r="4" spans="1:15" ht="16.5" customHeight="1">
       <c r="A4" s="144"/>
-      <c r="E4" s="220" t="s">
+      <c r="E4" s="210" t="s">
         <v>107</v>
       </c>
-      <c r="F4" s="221"/>
-      <c r="G4" s="221"/>
-      <c r="H4" s="221"/>
-      <c r="I4" s="221"/>
-      <c r="J4" s="221"/>
-      <c r="K4" s="221"/>
-      <c r="L4" s="222"/>
+      <c r="F4" s="211"/>
+      <c r="G4" s="211"/>
+      <c r="H4" s="211"/>
+      <c r="I4" s="211"/>
+      <c r="J4" s="211"/>
+      <c r="K4" s="211"/>
+      <c r="L4" s="212"/>
       <c r="O4" s="34"/>
     </row>
     <row r="5" spans="1:15" ht="16.5" customHeight="1">
       <c r="A5" s="144"/>
       <c r="D5" s="1"/>
-      <c r="E5" s="217" t="s">
+      <c r="E5" s="215" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="217"/>
-      <c r="G5" s="217" t="s">
+      <c r="F5" s="215"/>
+      <c r="G5" s="215" t="s">
         <v>31</v>
       </c>
-      <c r="H5" s="217"/>
-      <c r="I5" s="217" t="s">
+      <c r="H5" s="215"/>
+      <c r="I5" s="215" t="s">
         <v>32</v>
       </c>
-      <c r="J5" s="217"/>
-      <c r="K5" s="217" t="s">
+      <c r="J5" s="215"/>
+      <c r="K5" s="215" t="s">
         <v>83</v>
       </c>
-      <c r="L5" s="217"/>
+      <c r="L5" s="215"/>
       <c r="O5" s="34"/>
     </row>
     <row r="6" spans="1:15" ht="16.5" customHeight="1">
@@ -15554,10 +15558,10 @@
     </row>
     <row r="7" spans="1:15" ht="24" customHeight="1">
       <c r="A7" s="144"/>
-      <c r="B7" s="218" t="s">
+      <c r="B7" s="217" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="218"/>
+      <c r="C7" s="217"/>
       <c r="D7" s="38">
         <v>25</v>
       </c>
@@ -15573,10 +15577,10 @@
     </row>
     <row r="8" spans="1:15" ht="24" customHeight="1">
       <c r="A8" s="144"/>
-      <c r="B8" s="218" t="s">
+      <c r="B8" s="217" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="218"/>
+      <c r="C8" s="217"/>
       <c r="D8" s="38">
         <v>55</v>
       </c>
@@ -15592,10 +15596,10 @@
     </row>
     <row r="9" spans="1:15" ht="24" customHeight="1">
       <c r="A9" s="144"/>
-      <c r="B9" s="218" t="s">
+      <c r="B9" s="217" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="218"/>
+      <c r="C9" s="217"/>
       <c r="D9" s="38">
         <v>9</v>
       </c>
@@ -15611,10 +15615,10 @@
     </row>
     <row r="10" spans="1:15" ht="24" customHeight="1">
       <c r="A10" s="144"/>
-      <c r="B10" s="218" t="s">
+      <c r="B10" s="217" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="218"/>
+      <c r="C10" s="217"/>
       <c r="D10" s="38">
         <v>10</v>
       </c>
@@ -15630,10 +15634,10 @@
     </row>
     <row r="11" spans="1:15" ht="24" customHeight="1" thickBot="1">
       <c r="A11" s="144"/>
-      <c r="B11" s="218" t="s">
+      <c r="B11" s="217" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="218"/>
+      <c r="C11" s="217"/>
       <c r="D11" s="38">
         <v>100</v>
       </c>
@@ -15664,21 +15668,21 @@
     </row>
     <row r="14" spans="1:15" ht="18" customHeight="1">
       <c r="A14" s="144"/>
-      <c r="D14" s="219" t="s">
+      <c r="D14" s="230" t="s">
         <v>98</v>
       </c>
-      <c r="E14" s="219"/>
-      <c r="F14" s="219"/>
-      <c r="G14" s="219"/>
-      <c r="H14" s="219"/>
+      <c r="E14" s="230"/>
+      <c r="F14" s="230"/>
+      <c r="G14" s="230"/>
+      <c r="H14" s="230"/>
       <c r="I14" s="1"/>
-      <c r="J14" s="223" t="s">
+      <c r="J14" s="213" t="s">
         <v>99</v>
       </c>
-      <c r="K14" s="213" t="s">
+      <c r="K14" s="226" t="s">
         <v>107</v>
       </c>
-      <c r="L14" s="215" t="s">
+      <c r="L14" s="228" t="s">
         <v>41</v>
       </c>
       <c r="O14" s="34"/>
@@ -15701,17 +15705,17 @@
         <v>42</v>
       </c>
       <c r="I15" s="1"/>
-      <c r="J15" s="224"/>
-      <c r="K15" s="214"/>
-      <c r="L15" s="216"/>
+      <c r="J15" s="214"/>
+      <c r="K15" s="227"/>
+      <c r="L15" s="229"/>
       <c r="O15" s="34"/>
     </row>
     <row r="16" spans="1:15" ht="20.25" customHeight="1">
       <c r="A16" s="144"/>
-      <c r="B16" s="225" t="s">
+      <c r="B16" s="216" t="s">
         <v>43</v>
       </c>
-      <c r="C16" s="225"/>
+      <c r="C16" s="216"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
@@ -15728,10 +15732,10 @@
     </row>
     <row r="17" spans="1:15" ht="20.25" customHeight="1">
       <c r="A17" s="144"/>
-      <c r="B17" s="225" t="s">
+      <c r="B17" s="216" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="225"/>
+      <c r="C17" s="216"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -15748,10 +15752,10 @@
     </row>
     <row r="18" spans="1:15" ht="20.25" customHeight="1">
       <c r="A18" s="144"/>
-      <c r="B18" s="225" t="s">
+      <c r="B18" s="216" t="s">
         <v>45</v>
       </c>
-      <c r="C18" s="225"/>
+      <c r="C18" s="216"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
@@ -15768,10 +15772,10 @@
     </row>
     <row r="19" spans="1:15" ht="20.25" customHeight="1" thickBot="1">
       <c r="A19" s="144"/>
-      <c r="B19" s="225" t="s">
+      <c r="B19" s="216" t="s">
         <v>46</v>
       </c>
-      <c r="C19" s="225"/>
+      <c r="C19" s="216"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
@@ -15832,19 +15836,19 @@
       <c r="A23" s="144"/>
       <c r="B23" s="42"/>
       <c r="C23" s="42"/>
-      <c r="D23" s="228" t="s">
+      <c r="D23" s="220" t="s">
         <v>105</v>
       </c>
-      <c r="E23" s="228"/>
-      <c r="F23" s="228"/>
-      <c r="G23" s="228"/>
-      <c r="H23" s="228"/>
-      <c r="I23" s="228"/>
-      <c r="J23" s="228"/>
-      <c r="K23" s="228"/>
-      <c r="L23" s="228"/>
-      <c r="M23" s="228"/>
-      <c r="N23" s="210" t="s">
+      <c r="E23" s="220"/>
+      <c r="F23" s="220"/>
+      <c r="G23" s="220"/>
+      <c r="H23" s="220"/>
+      <c r="I23" s="220"/>
+      <c r="J23" s="220"/>
+      <c r="K23" s="220"/>
+      <c r="L23" s="220"/>
+      <c r="M23" s="220"/>
+      <c r="N23" s="223" t="s">
         <v>48</v>
       </c>
       <c r="O23" s="34"/>
@@ -15853,27 +15857,27 @@
       <c r="A24" s="144"/>
       <c r="B24" s="42"/>
       <c r="C24" s="42"/>
-      <c r="D24" s="218" t="s">
+      <c r="D24" s="217" t="s">
         <v>49</v>
       </c>
-      <c r="E24" s="218"/>
-      <c r="F24" s="218" t="s">
+      <c r="E24" s="217"/>
+      <c r="F24" s="217" t="s">
         <v>50</v>
       </c>
-      <c r="G24" s="218"/>
-      <c r="H24" s="218" t="s">
+      <c r="G24" s="217"/>
+      <c r="H24" s="217" t="s">
         <v>37</v>
       </c>
-      <c r="I24" s="218"/>
-      <c r="J24" s="218" t="s">
+      <c r="I24" s="217"/>
+      <c r="J24" s="217" t="s">
         <v>38</v>
       </c>
-      <c r="K24" s="218"/>
-      <c r="L24" s="218" t="s">
+      <c r="K24" s="217"/>
+      <c r="L24" s="217" t="s">
         <v>51</v>
       </c>
-      <c r="M24" s="218"/>
-      <c r="N24" s="210"/>
+      <c r="M24" s="217"/>
+      <c r="N24" s="223"/>
       <c r="O24" s="34"/>
     </row>
     <row r="25" spans="1:15" ht="26.25" customHeight="1">
@@ -15912,12 +15916,12 @@
       <c r="M25" s="47" t="s">
         <v>54</v>
       </c>
-      <c r="N25" s="210"/>
+      <c r="N25" s="223"/>
       <c r="O25" s="34"/>
     </row>
     <row r="26" spans="1:15" ht="18.75" customHeight="1">
       <c r="A26" s="144"/>
-      <c r="B26" s="226" t="s">
+      <c r="B26" s="218" t="s">
         <v>44</v>
       </c>
       <c r="C26" s="124">
@@ -15940,7 +15944,7 @@
     </row>
     <row r="27" spans="1:15" ht="18.75" customHeight="1">
       <c r="A27" s="144"/>
-      <c r="B27" s="227"/>
+      <c r="B27" s="219"/>
       <c r="C27" s="124">
         <v>17</v>
       </c>
@@ -15961,7 +15965,7 @@
     </row>
     <row r="28" spans="1:15" ht="18.75" customHeight="1">
       <c r="A28" s="144"/>
-      <c r="B28" s="217" t="s">
+      <c r="B28" s="215" t="s">
         <v>45</v>
       </c>
       <c r="C28" s="124">
@@ -15984,7 +15988,7 @@
     </row>
     <row r="29" spans="1:15" ht="18.75" customHeight="1">
       <c r="A29" s="144"/>
-      <c r="B29" s="217"/>
+      <c r="B29" s="215"/>
       <c r="C29" s="124">
         <v>17</v>
       </c>
@@ -16005,7 +16009,7 @@
     </row>
     <row r="30" spans="1:15" ht="18.75" customHeight="1">
       <c r="A30" s="144"/>
-      <c r="B30" s="217" t="s">
+      <c r="B30" s="215" t="s">
         <v>46</v>
       </c>
       <c r="C30" s="124">
@@ -16028,7 +16032,7 @@
     </row>
     <row r="31" spans="1:15" ht="18.75" customHeight="1">
       <c r="A31" s="144"/>
-      <c r="B31" s="217"/>
+      <c r="B31" s="215"/>
       <c r="C31" s="124">
         <v>17</v>
       </c>
@@ -16066,20 +16070,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="E4:L4"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D23:M23"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="N23:N25"/>
     <mergeCell ref="A1:B1"/>
@@ -16096,6 +16086,20 @@
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="D14:H14"/>
+    <mergeCell ref="E4:L4"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D23:M23"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>
@@ -16126,14 +16130,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="16.5" customHeight="1">
-      <c r="A1" s="211" t="s">
+      <c r="A1" s="224" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="212"/>
-      <c r="C1" s="208" t="s">
+      <c r="B1" s="225"/>
+      <c r="C1" s="221" t="s">
         <v>29</v>
       </c>
-      <c r="D1" s="209"/>
+      <c r="D1" s="222"/>
       <c r="E1" s="140"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
@@ -16165,37 +16169,37 @@
     </row>
     <row r="4" spans="1:15" ht="16.5" customHeight="1">
       <c r="A4" s="144"/>
-      <c r="E4" s="220" t="s">
+      <c r="E4" s="210" t="s">
         <v>107</v>
       </c>
-      <c r="F4" s="221"/>
-      <c r="G4" s="221"/>
-      <c r="H4" s="221"/>
-      <c r="I4" s="221"/>
-      <c r="J4" s="221"/>
-      <c r="K4" s="221"/>
-      <c r="L4" s="222"/>
+      <c r="F4" s="211"/>
+      <c r="G4" s="211"/>
+      <c r="H4" s="211"/>
+      <c r="I4" s="211"/>
+      <c r="J4" s="211"/>
+      <c r="K4" s="211"/>
+      <c r="L4" s="212"/>
       <c r="O4" s="34"/>
     </row>
     <row r="5" spans="1:15" ht="16.5" customHeight="1">
       <c r="A5" s="144"/>
       <c r="D5" s="1"/>
-      <c r="E5" s="217" t="s">
+      <c r="E5" s="215" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="217"/>
-      <c r="G5" s="217" t="s">
+      <c r="F5" s="215"/>
+      <c r="G5" s="215" t="s">
         <v>31</v>
       </c>
-      <c r="H5" s="217"/>
-      <c r="I5" s="217" t="s">
+      <c r="H5" s="215"/>
+      <c r="I5" s="215" t="s">
         <v>32</v>
       </c>
-      <c r="J5" s="217"/>
-      <c r="K5" s="217" t="s">
+      <c r="J5" s="215"/>
+      <c r="K5" s="215" t="s">
         <v>83</v>
       </c>
-      <c r="L5" s="217"/>
+      <c r="L5" s="215"/>
       <c r="O5" s="34"/>
     </row>
     <row r="6" spans="1:15" ht="16.5" customHeight="1">
@@ -16232,10 +16236,10 @@
     </row>
     <row r="7" spans="1:15" ht="24" customHeight="1">
       <c r="A7" s="144"/>
-      <c r="B7" s="218" t="s">
+      <c r="B7" s="217" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="218"/>
+      <c r="C7" s="217"/>
       <c r="D7" s="38">
         <v>25</v>
       </c>
@@ -16256,10 +16260,10 @@
     </row>
     <row r="8" spans="1:15" ht="24" customHeight="1">
       <c r="A8" s="144"/>
-      <c r="B8" s="218" t="s">
+      <c r="B8" s="217" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="218"/>
+      <c r="C8" s="217"/>
       <c r="D8" s="38">
         <v>55</v>
       </c>
@@ -16280,10 +16284,10 @@
     </row>
     <row r="9" spans="1:15" ht="24" customHeight="1">
       <c r="A9" s="144"/>
-      <c r="B9" s="218" t="s">
+      <c r="B9" s="217" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="218"/>
+      <c r="C9" s="217"/>
       <c r="D9" s="38">
         <v>9</v>
       </c>
@@ -16304,10 +16308,10 @@
     </row>
     <row r="10" spans="1:15" ht="24" customHeight="1">
       <c r="A10" s="144"/>
-      <c r="B10" s="218" t="s">
+      <c r="B10" s="217" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="218"/>
+      <c r="C10" s="217"/>
       <c r="D10" s="38">
         <v>10</v>
       </c>
@@ -16328,10 +16332,10 @@
     </row>
     <row r="11" spans="1:15" ht="24" customHeight="1" thickBot="1">
       <c r="A11" s="144"/>
-      <c r="B11" s="218" t="s">
+      <c r="B11" s="217" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="218"/>
+      <c r="C11" s="217"/>
       <c r="D11" s="38">
         <v>100</v>
       </c>
@@ -16370,21 +16374,21 @@
     </row>
     <row r="14" spans="1:15" ht="18" customHeight="1">
       <c r="A14" s="144"/>
-      <c r="D14" s="219" t="s">
+      <c r="D14" s="230" t="s">
         <v>98</v>
       </c>
-      <c r="E14" s="219"/>
-      <c r="F14" s="219"/>
-      <c r="G14" s="219"/>
-      <c r="H14" s="219"/>
+      <c r="E14" s="230"/>
+      <c r="F14" s="230"/>
+      <c r="G14" s="230"/>
+      <c r="H14" s="230"/>
       <c r="I14" s="1"/>
-      <c r="J14" s="223" t="s">
+      <c r="J14" s="213" t="s">
         <v>99</v>
       </c>
-      <c r="K14" s="213" t="s">
+      <c r="K14" s="226" t="s">
         <v>107</v>
       </c>
-      <c r="L14" s="215" t="s">
+      <c r="L14" s="228" t="s">
         <v>41</v>
       </c>
       <c r="O14" s="34"/>
@@ -16407,17 +16411,17 @@
         <v>42</v>
       </c>
       <c r="I15" s="1"/>
-      <c r="J15" s="224"/>
-      <c r="K15" s="214"/>
-      <c r="L15" s="216"/>
+      <c r="J15" s="214"/>
+      <c r="K15" s="227"/>
+      <c r="L15" s="229"/>
       <c r="O15" s="34"/>
     </row>
     <row r="16" spans="1:15" ht="20.25" customHeight="1">
       <c r="A16" s="144"/>
-      <c r="B16" s="225" t="s">
+      <c r="B16" s="216" t="s">
         <v>43</v>
       </c>
-      <c r="C16" s="225"/>
+      <c r="C16" s="216"/>
       <c r="D16" s="35">
         <v>0.75</v>
       </c>
@@ -16452,10 +16456,10 @@
     </row>
     <row r="17" spans="1:15" ht="20.25" customHeight="1">
       <c r="A17" s="144"/>
-      <c r="B17" s="225" t="s">
+      <c r="B17" s="216" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="225"/>
+      <c r="C17" s="216"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -16472,10 +16476,10 @@
     </row>
     <row r="18" spans="1:15" ht="20.25" customHeight="1">
       <c r="A18" s="144"/>
-      <c r="B18" s="225" t="s">
+      <c r="B18" s="216" t="s">
         <v>45</v>
       </c>
-      <c r="C18" s="225"/>
+      <c r="C18" s="216"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
@@ -16492,10 +16496,10 @@
     </row>
     <row r="19" spans="1:15" ht="20.25" customHeight="1" thickBot="1">
       <c r="A19" s="144"/>
-      <c r="B19" s="225" t="s">
+      <c r="B19" s="216" t="s">
         <v>46</v>
       </c>
-      <c r="C19" s="225"/>
+      <c r="C19" s="216"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
@@ -16556,19 +16560,19 @@
       <c r="A23" s="144"/>
       <c r="B23" s="42"/>
       <c r="C23" s="42"/>
-      <c r="D23" s="228" t="s">
+      <c r="D23" s="220" t="s">
         <v>105</v>
       </c>
-      <c r="E23" s="228"/>
-      <c r="F23" s="228"/>
-      <c r="G23" s="228"/>
-      <c r="H23" s="228"/>
-      <c r="I23" s="228"/>
-      <c r="J23" s="228"/>
-      <c r="K23" s="228"/>
-      <c r="L23" s="228"/>
-      <c r="M23" s="228"/>
-      <c r="N23" s="210" t="s">
+      <c r="E23" s="220"/>
+      <c r="F23" s="220"/>
+      <c r="G23" s="220"/>
+      <c r="H23" s="220"/>
+      <c r="I23" s="220"/>
+      <c r="J23" s="220"/>
+      <c r="K23" s="220"/>
+      <c r="L23" s="220"/>
+      <c r="M23" s="220"/>
+      <c r="N23" s="223" t="s">
         <v>48</v>
       </c>
       <c r="O23" s="34"/>
@@ -16577,27 +16581,27 @@
       <c r="A24" s="144"/>
       <c r="B24" s="42"/>
       <c r="C24" s="42"/>
-      <c r="D24" s="218" t="s">
+      <c r="D24" s="217" t="s">
         <v>49</v>
       </c>
-      <c r="E24" s="218"/>
-      <c r="F24" s="218" t="s">
+      <c r="E24" s="217"/>
+      <c r="F24" s="217" t="s">
         <v>50</v>
       </c>
-      <c r="G24" s="218"/>
-      <c r="H24" s="218" t="s">
+      <c r="G24" s="217"/>
+      <c r="H24" s="217" t="s">
         <v>37</v>
       </c>
-      <c r="I24" s="218"/>
-      <c r="J24" s="218" t="s">
+      <c r="I24" s="217"/>
+      <c r="J24" s="217" t="s">
         <v>38</v>
       </c>
-      <c r="K24" s="218"/>
-      <c r="L24" s="218" t="s">
+      <c r="K24" s="217"/>
+      <c r="L24" s="217" t="s">
         <v>51</v>
       </c>
-      <c r="M24" s="218"/>
-      <c r="N24" s="210"/>
+      <c r="M24" s="217"/>
+      <c r="N24" s="223"/>
       <c r="O24" s="34"/>
     </row>
     <row r="25" spans="1:15" ht="26.25" customHeight="1">
@@ -16636,12 +16640,12 @@
       <c r="M25" s="47" t="s">
         <v>54</v>
       </c>
-      <c r="N25" s="210"/>
+      <c r="N25" s="223"/>
       <c r="O25" s="34"/>
     </row>
     <row r="26" spans="1:15" ht="18.75" customHeight="1">
       <c r="A26" s="144"/>
-      <c r="B26" s="226" t="s">
+      <c r="B26" s="218" t="s">
         <v>44</v>
       </c>
       <c r="C26" s="124">
@@ -16668,7 +16672,7 @@
     </row>
     <row r="27" spans="1:15" ht="18.75" customHeight="1">
       <c r="A27" s="144"/>
-      <c r="B27" s="227"/>
+      <c r="B27" s="219"/>
       <c r="C27" s="124">
         <v>17</v>
       </c>
@@ -16691,7 +16695,7 @@
     </row>
     <row r="28" spans="1:15" ht="18.75" customHeight="1">
       <c r="A28" s="144"/>
-      <c r="B28" s="217" t="s">
+      <c r="B28" s="215" t="s">
         <v>45</v>
       </c>
       <c r="C28" s="124">
@@ -16720,7 +16724,7 @@
     </row>
     <row r="29" spans="1:15" ht="18.75" customHeight="1">
       <c r="A29" s="144"/>
-      <c r="B29" s="217"/>
+      <c r="B29" s="215"/>
       <c r="C29" s="124">
         <v>17</v>
       </c>
@@ -16745,7 +16749,7 @@
     </row>
     <row r="30" spans="1:15" ht="18.75" customHeight="1">
       <c r="A30" s="144"/>
-      <c r="B30" s="217" t="s">
+      <c r="B30" s="215" t="s">
         <v>46</v>
       </c>
       <c r="C30" s="124">
@@ -16776,7 +16780,7 @@
     </row>
     <row r="31" spans="1:15" ht="18.75" customHeight="1">
       <c r="A31" s="144"/>
-      <c r="B31" s="217"/>
+      <c r="B31" s="215"/>
       <c r="C31" s="124">
         <v>17</v>
       </c>
@@ -16822,20 +16826,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="K14:K15"/>
-    <mergeCell ref="L14:L15"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="E4:L4"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="N23:N25"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="L24:M24"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J14:J15"/>
     <mergeCell ref="B30:B31"/>
     <mergeCell ref="B28:B29"/>
     <mergeCell ref="I5:J5"/>
@@ -16852,6 +16842,20 @@
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B10:C10"/>
+    <mergeCell ref="N23:N25"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="E4:L4"/>
+    <mergeCell ref="B9:C9"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>
@@ -16892,24 +16896,24 @@
     <row r="3" spans="1:14" ht="16.5" customHeight="1">
       <c r="A3" s="42"/>
       <c r="B3" s="42"/>
-      <c r="C3" s="234" t="s">
+      <c r="C3" s="240" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="234"/>
-      <c r="E3" s="234"/>
-      <c r="F3" s="234"/>
-      <c r="G3" s="234"/>
-      <c r="H3" s="234"/>
-      <c r="I3" s="234"/>
-      <c r="J3" s="234"/>
-      <c r="K3" s="234"/>
-      <c r="L3" s="234"/>
+      <c r="D3" s="240"/>
+      <c r="E3" s="240"/>
+      <c r="F3" s="240"/>
+      <c r="G3" s="240"/>
+      <c r="H3" s="240"/>
+      <c r="I3" s="240"/>
+      <c r="J3" s="240"/>
+      <c r="K3" s="240"/>
+      <c r="L3" s="240"/>
     </row>
     <row r="4" spans="1:14" ht="24" customHeight="1">
-      <c r="A4" s="229" t="s">
+      <c r="A4" s="238" t="s">
         <v>109</v>
       </c>
-      <c r="B4" s="230"/>
+      <c r="B4" s="239"/>
       <c r="C4" s="233" t="s">
         <v>84</v>
       </c>
@@ -17095,10 +17099,10 @@
     </row>
     <row r="12" spans="1:14" ht="16.5" customHeight="1"/>
     <row r="13" spans="1:14" ht="21.75" customHeight="1">
-      <c r="A13" s="237" t="s">
+      <c r="A13" s="236" t="s">
         <v>111</v>
       </c>
-      <c r="B13" s="238"/>
+      <c r="B13" s="237"/>
       <c r="C13" s="233" t="s">
         <v>84</v>
       </c>
@@ -17283,10 +17287,10 @@
     </row>
     <row r="21" spans="1:13" ht="13.5" customHeight="1"/>
     <row r="22" spans="1:13" ht="21.75" customHeight="1">
-      <c r="A22" s="235" t="s">
+      <c r="A22" s="234" t="s">
         <v>112</v>
       </c>
-      <c r="B22" s="236"/>
+      <c r="B22" s="235"/>
       <c r="C22" s="233" t="s">
         <v>84</v>
       </c>
@@ -17471,11 +17475,14 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C3:L3"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="E4:F4"/>
     <mergeCell ref="A10:A11"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="K22:L22"/>
@@ -17491,14 +17498,11 @@
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="G13:H13"/>
     <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C3:L3"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="I22:J22"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>
@@ -17537,21 +17541,21 @@
       </c>
     </row>
     <row r="2" spans="2:10" ht="17.25" customHeight="1">
-      <c r="F2" s="242" t="s">
+      <c r="F2" s="244" t="s">
         <v>71</v>
       </c>
-      <c r="G2" s="243"/>
-      <c r="H2" s="243"/>
-      <c r="I2" s="244"/>
+      <c r="G2" s="245"/>
+      <c r="H2" s="245"/>
+      <c r="I2" s="246"/>
     </row>
     <row r="3" spans="2:10" ht="27" customHeight="1">
-      <c r="B3" s="239" t="s">
+      <c r="B3" s="241" t="s">
         <v>72</v>
       </c>
-      <c r="C3" s="245" t="s">
+      <c r="C3" s="247" t="s">
         <v>64</v>
       </c>
-      <c r="D3" s="246"/>
+      <c r="D3" s="248"/>
       <c r="F3" s="37" t="s">
         <v>65</v>
       </c>
@@ -17566,7 +17570,7 @@
       </c>
     </row>
     <row r="4" spans="2:10" ht="16.5" customHeight="1">
-      <c r="B4" s="240"/>
+      <c r="B4" s="242"/>
       <c r="C4" s="72" t="s">
         <v>70</v>
       </c>
@@ -17589,7 +17593,7 @@
       </c>
     </row>
     <row r="5" spans="2:10" ht="18" customHeight="1">
-      <c r="B5" s="240"/>
+      <c r="B5" s="242"/>
       <c r="C5" s="98" t="s">
         <v>44</v>
       </c>
@@ -17600,7 +17604,7 @@
       <c r="I5" s="85"/>
     </row>
     <row r="6" spans="2:10" ht="18" customHeight="1">
-      <c r="B6" s="240"/>
+      <c r="B6" s="242"/>
       <c r="C6" s="99" t="s">
         <v>45</v>
       </c>
@@ -17611,7 +17615,7 @@
       <c r="I6" s="89"/>
     </row>
     <row r="7" spans="2:10" ht="18" customHeight="1">
-      <c r="B7" s="240"/>
+      <c r="B7" s="242"/>
       <c r="C7" s="100" t="s">
         <v>46</v>
       </c>
@@ -17625,7 +17629,7 @@
       </c>
     </row>
     <row r="8" spans="2:10" ht="18" customHeight="1">
-      <c r="B8" s="241"/>
+      <c r="B8" s="243"/>
       <c r="C8" s="94" t="s">
         <v>82</v>
       </c>
@@ -17652,21 +17656,21 @@
     <row r="10" spans="2:10" ht="15" customHeight="1">
       <c r="B10" s="2"/>
       <c r="D10" s="97"/>
-      <c r="F10" s="242" t="s">
+      <c r="F10" s="244" t="s">
         <v>71</v>
       </c>
-      <c r="G10" s="243"/>
-      <c r="H10" s="243"/>
-      <c r="I10" s="244"/>
+      <c r="G10" s="245"/>
+      <c r="H10" s="245"/>
+      <c r="I10" s="246"/>
     </row>
     <row r="11" spans="2:10" ht="27" customHeight="1">
-      <c r="B11" s="239" t="s">
+      <c r="B11" s="241" t="s">
         <v>73</v>
       </c>
-      <c r="C11" s="245" t="s">
+      <c r="C11" s="247" t="s">
         <v>64</v>
       </c>
-      <c r="D11" s="246"/>
+      <c r="D11" s="248"/>
       <c r="F11" s="3" t="s">
         <v>66</v>
       </c>
@@ -17681,7 +17685,7 @@
       </c>
     </row>
     <row r="12" spans="2:10" ht="16.5" customHeight="1">
-      <c r="B12" s="240"/>
+      <c r="B12" s="242"/>
       <c r="C12" s="72" t="s">
         <v>70</v>
       </c>
@@ -17704,7 +17708,7 @@
       </c>
     </row>
     <row r="13" spans="2:10" ht="18" customHeight="1">
-      <c r="B13" s="240"/>
+      <c r="B13" s="242"/>
       <c r="C13" s="98" t="s">
         <v>44</v>
       </c>
@@ -17715,7 +17719,7 @@
       <c r="I13" s="85"/>
     </row>
     <row r="14" spans="2:10" ht="18" customHeight="1">
-      <c r="B14" s="240"/>
+      <c r="B14" s="242"/>
       <c r="C14" s="99" t="s">
         <v>45</v>
       </c>
@@ -17726,7 +17730,7 @@
       <c r="I14" s="89"/>
     </row>
     <row r="15" spans="2:10" ht="18" customHeight="1">
-      <c r="B15" s="240"/>
+      <c r="B15" s="242"/>
       <c r="C15" s="100" t="s">
         <v>46</v>
       </c>
@@ -17740,7 +17744,7 @@
       </c>
     </row>
     <row r="16" spans="2:10" ht="18" customHeight="1">
-      <c r="B16" s="241"/>
+      <c r="B16" s="243"/>
       <c r="C16" s="94" t="s">
         <v>82</v>
       </c>
@@ -17767,21 +17771,21 @@
     <row r="18" spans="2:10" ht="14.25" customHeight="1">
       <c r="B18" s="2"/>
       <c r="D18" s="97"/>
-      <c r="F18" s="242" t="s">
+      <c r="F18" s="244" t="s">
         <v>71</v>
       </c>
-      <c r="G18" s="243"/>
-      <c r="H18" s="243"/>
-      <c r="I18" s="244"/>
+      <c r="G18" s="245"/>
+      <c r="H18" s="245"/>
+      <c r="I18" s="246"/>
     </row>
     <row r="19" spans="2:10" ht="27" customHeight="1">
-      <c r="B19" s="239" t="s">
+      <c r="B19" s="241" t="s">
         <v>74</v>
       </c>
-      <c r="C19" s="245" t="s">
+      <c r="C19" s="247" t="s">
         <v>64</v>
       </c>
-      <c r="D19" s="246"/>
+      <c r="D19" s="248"/>
       <c r="F19" s="37" t="s">
         <v>67</v>
       </c>
@@ -17796,7 +17800,7 @@
       </c>
     </row>
     <row r="20" spans="2:10" ht="18" customHeight="1">
-      <c r="B20" s="240"/>
+      <c r="B20" s="242"/>
       <c r="C20" s="72" t="s">
         <v>70</v>
       </c>
@@ -17819,7 +17823,7 @@
       </c>
     </row>
     <row r="21" spans="2:10" ht="18" customHeight="1">
-      <c r="B21" s="240"/>
+      <c r="B21" s="242"/>
       <c r="C21" s="98" t="s">
         <v>44</v>
       </c>
@@ -17830,7 +17834,7 @@
       <c r="I21" s="85"/>
     </row>
     <row r="22" spans="2:10" ht="18" customHeight="1">
-      <c r="B22" s="240"/>
+      <c r="B22" s="242"/>
       <c r="C22" s="99" t="s">
         <v>45</v>
       </c>
@@ -17841,7 +17845,7 @@
       <c r="I22" s="89"/>
     </row>
     <row r="23" spans="2:10" ht="18" customHeight="1">
-      <c r="B23" s="240"/>
+      <c r="B23" s="242"/>
       <c r="C23" s="100" t="s">
         <v>46</v>
       </c>
@@ -17855,7 +17859,7 @@
       </c>
     </row>
     <row r="24" spans="2:10" ht="18" customHeight="1">
-      <c r="B24" s="241"/>
+      <c r="B24" s="243"/>
       <c r="C24" s="94" t="s">
         <v>82</v>
       </c>
@@ -17929,21 +17933,21 @@
       </c>
     </row>
     <row r="2" spans="2:10" ht="17.25" customHeight="1">
-      <c r="F2" s="242" t="s">
+      <c r="F2" s="244" t="s">
         <v>71</v>
       </c>
-      <c r="G2" s="243"/>
-      <c r="H2" s="243"/>
-      <c r="I2" s="244"/>
+      <c r="G2" s="245"/>
+      <c r="H2" s="245"/>
+      <c r="I2" s="246"/>
     </row>
     <row r="3" spans="2:10" ht="27" customHeight="1">
-      <c r="B3" s="239" t="s">
+      <c r="B3" s="241" t="s">
         <v>72</v>
       </c>
-      <c r="C3" s="245" t="s">
+      <c r="C3" s="247" t="s">
         <v>64</v>
       </c>
-      <c r="D3" s="246"/>
+      <c r="D3" s="248"/>
       <c r="F3" s="37" t="s">
         <v>65</v>
       </c>
@@ -17958,7 +17962,7 @@
       </c>
     </row>
     <row r="4" spans="2:10" ht="16.5" customHeight="1">
-      <c r="B4" s="240"/>
+      <c r="B4" s="242"/>
       <c r="C4" s="72" t="s">
         <v>70</v>
       </c>
@@ -17981,7 +17985,7 @@
       </c>
     </row>
     <row r="5" spans="2:10" ht="18" customHeight="1">
-      <c r="B5" s="240"/>
+      <c r="B5" s="242"/>
       <c r="C5" s="98" t="s">
         <v>44</v>
       </c>
@@ -17994,7 +17998,7 @@
       <c r="I5" s="85"/>
     </row>
     <row r="6" spans="2:10" ht="18" customHeight="1">
-      <c r="B6" s="240"/>
+      <c r="B6" s="242"/>
       <c r="C6" s="99" t="s">
         <v>45</v>
       </c>
@@ -18007,7 +18011,7 @@
       <c r="I6" s="89"/>
     </row>
     <row r="7" spans="2:10" ht="18" customHeight="1">
-      <c r="B7" s="240"/>
+      <c r="B7" s="242"/>
       <c r="C7" s="100" t="s">
         <v>46</v>
       </c>
@@ -18023,7 +18027,7 @@
       </c>
     </row>
     <row r="8" spans="2:10" ht="18" customHeight="1">
-      <c r="B8" s="241"/>
+      <c r="B8" s="243"/>
       <c r="C8" s="94" t="s">
         <v>82</v>
       </c>
@@ -18061,21 +18065,21 @@
     <row r="10" spans="2:10" ht="15" customHeight="1">
       <c r="B10" s="2"/>
       <c r="D10" s="97"/>
-      <c r="F10" s="242" t="s">
+      <c r="F10" s="244" t="s">
         <v>71</v>
       </c>
-      <c r="G10" s="243"/>
-      <c r="H10" s="243"/>
-      <c r="I10" s="244"/>
+      <c r="G10" s="245"/>
+      <c r="H10" s="245"/>
+      <c r="I10" s="246"/>
     </row>
     <row r="11" spans="2:10" ht="27" customHeight="1">
-      <c r="B11" s="239" t="s">
+      <c r="B11" s="241" t="s">
         <v>73</v>
       </c>
-      <c r="C11" s="245" t="s">
+      <c r="C11" s="247" t="s">
         <v>64</v>
       </c>
-      <c r="D11" s="246"/>
+      <c r="D11" s="248"/>
       <c r="F11" s="3" t="s">
         <v>66</v>
       </c>
@@ -18090,7 +18094,7 @@
       </c>
     </row>
     <row r="12" spans="2:10" ht="16.5" customHeight="1">
-      <c r="B12" s="240"/>
+      <c r="B12" s="242"/>
       <c r="C12" s="72" t="s">
         <v>70</v>
       </c>
@@ -18113,7 +18117,7 @@
       </c>
     </row>
     <row r="13" spans="2:10" ht="18" customHeight="1">
-      <c r="B13" s="240"/>
+      <c r="B13" s="242"/>
       <c r="C13" s="98" t="s">
         <v>44</v>
       </c>
@@ -18126,7 +18130,7 @@
       <c r="I13" s="85"/>
     </row>
     <row r="14" spans="2:10" ht="18" customHeight="1">
-      <c r="B14" s="240"/>
+      <c r="B14" s="242"/>
       <c r="C14" s="99" t="s">
         <v>45</v>
       </c>
@@ -18139,7 +18143,7 @@
       <c r="I14" s="89"/>
     </row>
     <row r="15" spans="2:10" ht="18" customHeight="1">
-      <c r="B15" s="240"/>
+      <c r="B15" s="242"/>
       <c r="C15" s="100" t="s">
         <v>46</v>
       </c>
@@ -18155,7 +18159,7 @@
       </c>
     </row>
     <row r="16" spans="2:10" ht="18" customHeight="1">
-      <c r="B16" s="241"/>
+      <c r="B16" s="243"/>
       <c r="C16" s="94" t="s">
         <v>82</v>
       </c>
@@ -18193,21 +18197,21 @@
     <row r="18" spans="2:10" ht="14.25" customHeight="1">
       <c r="B18" s="2"/>
       <c r="D18" s="97"/>
-      <c r="F18" s="242" t="s">
+      <c r="F18" s="244" t="s">
         <v>71</v>
       </c>
-      <c r="G18" s="243"/>
-      <c r="H18" s="243"/>
-      <c r="I18" s="244"/>
+      <c r="G18" s="245"/>
+      <c r="H18" s="245"/>
+      <c r="I18" s="246"/>
     </row>
     <row r="19" spans="2:10" ht="27" customHeight="1">
-      <c r="B19" s="239" t="s">
+      <c r="B19" s="241" t="s">
         <v>74</v>
       </c>
-      <c r="C19" s="245" t="s">
+      <c r="C19" s="247" t="s">
         <v>64</v>
       </c>
-      <c r="D19" s="246"/>
+      <c r="D19" s="248"/>
       <c r="F19" s="37" t="s">
         <v>67</v>
       </c>
@@ -18222,7 +18226,7 @@
       </c>
     </row>
     <row r="20" spans="2:10" ht="18" customHeight="1">
-      <c r="B20" s="240"/>
+      <c r="B20" s="242"/>
       <c r="C20" s="72" t="s">
         <v>70</v>
       </c>
@@ -18245,7 +18249,7 @@
       </c>
     </row>
     <row r="21" spans="2:10" ht="18" customHeight="1">
-      <c r="B21" s="240"/>
+      <c r="B21" s="242"/>
       <c r="C21" s="98" t="s">
         <v>44</v>
       </c>
@@ -18258,7 +18262,7 @@
       <c r="I21" s="85"/>
     </row>
     <row r="22" spans="2:10" ht="18" customHeight="1">
-      <c r="B22" s="240"/>
+      <c r="B22" s="242"/>
       <c r="C22" s="99" t="s">
         <v>45</v>
       </c>
@@ -18271,7 +18275,7 @@
       <c r="I22" s="89"/>
     </row>
     <row r="23" spans="2:10" ht="18" customHeight="1">
-      <c r="B23" s="240"/>
+      <c r="B23" s="242"/>
       <c r="C23" s="100" t="s">
         <v>46</v>
       </c>
@@ -18287,7 +18291,7 @@
       </c>
     </row>
     <row r="24" spans="2:10" ht="18" customHeight="1">
-      <c r="B24" s="241"/>
+      <c r="B24" s="243"/>
       <c r="C24" s="94" t="s">
         <v>82</v>
       </c>

</xml_diff>